<commit_message>
switch to family office workspace
</commit_message>
<xml_diff>
--- a/workspace/sheets/budget_vs_actual_2026.xlsx
+++ b/workspace/sheets/budget_vs_actual_2026.xlsx
@@ -440,11 +440,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -455,14 +455,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Harbour Lane Trading Ltd - Budget vs Actual 2026, YTD Jan-Sep</t>
+          <t>Lantau Peak Family Office Ltd - Budget vs Actual 2026, YTD Jan-Sep</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Budget approved by D. Wong 20 Jan 2026. Actuals from GL export. Variance = Actual - Budget (expenses: positive = over budget).</t>
+          <t>Budget approved by V. Cheung 20 Jan 2026. Actuals from GL export. Variance = Actual - Budget (expenses: positive = over budget).</t>
         </is>
       </c>
     </row>
@@ -506,24 +506,24 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>260</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Rental Income</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Income</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>12150000</v>
+        <v>1413000</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>12477460</v>
+        <v>1413000</v>
       </c>
       <c r="F5" s="3">
         <f>E5-D5</f>
@@ -537,24 +537,24 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>270</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Other Revenue</t>
+          <t>Interest Income</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Income</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0</v>
+        <v>765000</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0</v>
+        <v>703785</v>
       </c>
       <c r="F6" s="3">
         <f>E6-D6</f>
@@ -568,24 +568,24 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>275</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Interest Income</t>
+          <t>Dividend &amp; Portfolio Income</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Income</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>13500</v>
+        <v>34200000</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>12613</v>
+        <v>33340000</v>
       </c>
       <c r="F7" s="3">
         <f>E7-D7</f>
@@ -599,24 +599,24 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>477</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold</t>
+          <t>Salaries - Office &amp; Household Staff</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Cost of sales</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>5400000</v>
+        <v>3780000</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>5536128.36</v>
+        <v>3780000</v>
       </c>
       <c r="F8" s="3">
         <f>E8-D8</f>
@@ -630,24 +630,24 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>425</t>
+          <t>478</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Freight &amp; Courier</t>
+          <t>MPF Contributions</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Freight &amp; logistics</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>162000</v>
+        <v>135000</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>190275</v>
+        <v>135000</v>
       </c>
       <c r="F9" s="3">
         <f>E9-D9</f>
@@ -661,24 +661,24 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>445</t>
+          <t>471</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Utilities - Electricity</t>
+          <t>Property Management Fees</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Facilities</t>
+          <t>Property</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>43200</v>
+        <v>162000</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>44672</v>
+        <v>191100</v>
       </c>
       <c r="F10" s="3">
         <f>E10-D10</f>
@@ -692,24 +692,24 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>469</t>
+          <t>473</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Rent</t>
+          <t>Property Repairs &amp; Maintenance</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Facilities</t>
+          <t>Property</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>720000</v>
+        <v>27000</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>744000</v>
+        <v>65300</v>
       </c>
       <c r="F11" s="3">
         <f>E11-D11</f>
@@ -723,24 +723,24 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>471</t>
+          <t>475</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Building Management Fees</t>
+          <t>Building Management &amp; Government Rates</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Facilities</t>
+          <t>Property</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>61200</v>
+        <v>104400</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>66000</v>
+        <v>109200</v>
       </c>
       <c r="F12" s="3">
         <f>E12-D12</f>
@@ -754,24 +754,24 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>473</t>
+          <t>481</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>School &amp; Tuition Fees</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Facilities</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>18000</v>
+        <v>598000</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>61500</v>
+        <v>604000</v>
       </c>
       <c r="F13" s="3">
         <f>E13-D13</f>
@@ -785,24 +785,24 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>477</t>
+          <t>493</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Salaries</t>
+          <t>Travel &amp; Aviation Charter</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>Travel &amp; aviation</t>
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>3888000</v>
+        <v>1125000</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>3888000</v>
+        <v>1127000</v>
       </c>
       <c r="F14" s="3">
         <f>E14-D14</f>
@@ -816,24 +816,24 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>478</t>
+          <t>433</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MPF Contributions</t>
+          <t>Insurance</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>Insurance</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>237600</v>
+        <v>219000</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>237600</v>
+        <v>220112.5</v>
       </c>
       <c r="F15" s="3">
         <f>E15-D15</f>
@@ -847,24 +847,24 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>412</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Bank Fees</t>
+          <t>Legal, Tax &amp; Audit Fees</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Professional fees</t>
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>4050</v>
+        <v>372000</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>5130</v>
+        <v>372000</v>
       </c>
       <c r="F16" s="3">
         <f>E16-D16</f>
@@ -878,24 +878,24 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>412</t>
+          <t>455</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Consulting &amp; Accounting</t>
+          <t>Fund Management Fees</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Fund fees</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>45000</v>
+        <v>877500</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>45000</v>
+        <v>877875</v>
       </c>
       <c r="F17" s="3">
         <f>E17-D17</f>
@@ -909,12 +909,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>429</t>
+          <t>404</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>General Expenses</t>
+          <t>Bank Fees</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -923,10 +923,10 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>22500</v>
+        <v>8100</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>18100</v>
+        <v>3930</v>
       </c>
       <c r="F18" s="3">
         <f>E18-D18</f>
@@ -940,12 +940,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>433</t>
+          <t>429</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Insurance</t>
+          <t>General Office Expenses</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -954,10 +954,10 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>28800</v>
+        <v>81000</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>28800</v>
+        <v>78000</v>
       </c>
       <c r="F19" s="3">
         <f>E19-D19</f>
@@ -985,10 +985,10 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>114300</v>
+        <v>28800</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>113742.5</v>
+        <v>28350</v>
       </c>
       <c r="F20" s="3">
         <f>E20-D20</f>
@@ -1016,10 +1016,10 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>17100</v>
+        <v>21600</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>16920</v>
+        <v>21420</v>
       </c>
       <c r="F21" s="3">
         <f>E21-D21</f>
@@ -1033,12 +1033,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>493</t>
+          <t>497</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Travel - Local &amp; Cross-border</t>
+          <t>Foreign Exchange Gain/Loss</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1047,10 +1047,10 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>36000</v>
+        <v>0</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>28800</v>
+        <v>375</v>
       </c>
       <c r="F22" s="3">
         <f>E22-D22</f>
@@ -1062,58 +1062,56 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>497</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Foreign Exchange Gain/Loss</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Admin</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="3" t="n">
-        <v>6032.44</v>
-      </c>
-      <c r="F23" s="3">
-        <f>E23-D23</f>
-        <v/>
-      </c>
-      <c r="G23" s="4">
-        <f>IF(D23=0,"",F23/D23)</f>
-        <v/>
-      </c>
+      <c r="D23" s="3" t="n"/>
+      <c r="E23" s="3" t="n"/>
+      <c r="F23" s="3" t="n"/>
+      <c r="G23" s="4" t="n"/>
     </row>
     <row r="24">
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>By group</t>
+        </is>
+      </c>
       <c r="D24" s="3" t="n"/>
       <c r="E24" s="3" t="n"/>
       <c r="F24" s="3" t="n"/>
       <c r="G24" s="4" t="n"/>
     </row>
     <row r="25">
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>By group</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
-      <c r="G25" s="4" t="n"/>
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>group total</t>
+        </is>
+      </c>
+      <c r="D25" s="3">
+        <f>SUMIF($C$5:$C$22,B25,D$5:D$22)</f>
+        <v/>
+      </c>
+      <c r="E25" s="3">
+        <f>SUMIF($C$5:$C$22,B25,E$5:E$22)</f>
+        <v/>
+      </c>
+      <c r="F25" s="3">
+        <f>E25-D25</f>
+        <v/>
+      </c>
+      <c r="G25" s="4">
+        <f>IF(D25=0,"",F25/D25)</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1122,11 +1120,11 @@
         </is>
       </c>
       <c r="D26" s="3">
-        <f>SUMIF($C$5:$C$23,B26,D$5:D$23)</f>
+        <f>SUMIF($C$5:$C$22,B26,D$5:D$22)</f>
         <v/>
       </c>
       <c r="E26" s="3">
-        <f>SUMIF($C$5:$C$23,B26,E$5:E$23)</f>
+        <f>SUMIF($C$5:$C$22,B26,E$5:E$22)</f>
         <v/>
       </c>
       <c r="F26" s="3">
@@ -1142,7 +1140,7 @@
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Cost of sales</t>
+          <t>Property</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1151,11 +1149,11 @@
         </is>
       </c>
       <c r="D27" s="3">
-        <f>SUMIF($C$5:$C$23,B27,D$5:D$23)</f>
+        <f>SUMIF($C$5:$C$22,B27,D$5:D$22)</f>
         <v/>
       </c>
       <c r="E27" s="3">
-        <f>SUMIF($C$5:$C$23,B27,E$5:E$23)</f>
+        <f>SUMIF($C$5:$C$22,B27,E$5:E$22)</f>
         <v/>
       </c>
       <c r="F27" s="3">
@@ -1171,7 +1169,7 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Freight &amp; logistics</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1180,11 +1178,11 @@
         </is>
       </c>
       <c r="D28" s="3">
-        <f>SUMIF($C$5:$C$23,B28,D$5:D$23)</f>
+        <f>SUMIF($C$5:$C$22,B28,D$5:D$22)</f>
         <v/>
       </c>
       <c r="E28" s="3">
-        <f>SUMIF($C$5:$C$23,B28,E$5:E$23)</f>
+        <f>SUMIF($C$5:$C$22,B28,E$5:E$22)</f>
         <v/>
       </c>
       <c r="F28" s="3">
@@ -1200,7 +1198,7 @@
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Facilities</t>
+          <t>Travel &amp; aviation</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1209,11 +1207,11 @@
         </is>
       </c>
       <c r="D29" s="3">
-        <f>SUMIF($C$5:$C$23,B29,D$5:D$23)</f>
+        <f>SUMIF($C$5:$C$22,B29,D$5:D$22)</f>
         <v/>
       </c>
       <c r="E29" s="3">
-        <f>SUMIF($C$5:$C$23,B29,E$5:E$23)</f>
+        <f>SUMIF($C$5:$C$22,B29,E$5:E$22)</f>
         <v/>
       </c>
       <c r="F29" s="3">
@@ -1229,7 +1227,7 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>Insurance</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1238,11 +1236,11 @@
         </is>
       </c>
       <c r="D30" s="3">
-        <f>SUMIF($C$5:$C$23,B30,D$5:D$23)</f>
+        <f>SUMIF($C$5:$C$22,B30,D$5:D$22)</f>
         <v/>
       </c>
       <c r="E30" s="3">
-        <f>SUMIF($C$5:$C$23,B30,E$5:E$23)</f>
+        <f>SUMIF($C$5:$C$22,B30,E$5:E$22)</f>
         <v/>
       </c>
       <c r="F30" s="3">
@@ -1258,7 +1256,7 @@
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Professional fees</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1267,11 +1265,11 @@
         </is>
       </c>
       <c r="D31" s="3">
-        <f>SUMIF($C$5:$C$23,B31,D$5:D$23)</f>
+        <f>SUMIF($C$5:$C$22,B31,D$5:D$22)</f>
         <v/>
       </c>
       <c r="E31" s="3">
-        <f>SUMIF($C$5:$C$23,B31,E$5:E$23)</f>
+        <f>SUMIF($C$5:$C$22,B31,E$5:E$22)</f>
         <v/>
       </c>
       <c r="F31" s="3">
@@ -1280,6 +1278,64 @@
       </c>
       <c r="G31" s="4">
         <f>IF(D31=0,"",F31/D31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Fund fees</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>group total</t>
+        </is>
+      </c>
+      <c r="D32" s="3">
+        <f>SUMIF($C$5:$C$22,B32,D$5:D$22)</f>
+        <v/>
+      </c>
+      <c r="E32" s="3">
+        <f>SUMIF($C$5:$C$22,B32,E$5:E$22)</f>
+        <v/>
+      </c>
+      <c r="F32" s="3">
+        <f>E32-D32</f>
+        <v/>
+      </c>
+      <c r="G32" s="4">
+        <f>IF(D32=0,"",F32/D32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>group total</t>
+        </is>
+      </c>
+      <c r="D33" s="3">
+        <f>SUMIF($C$5:$C$22,B33,D$5:D$22)</f>
+        <v/>
+      </c>
+      <c r="E33" s="3">
+        <f>SUMIF($C$5:$C$22,B33,E$5:E$22)</f>
+        <v/>
+      </c>
+      <c r="F33" s="3">
+        <f>E33-D33</f>
+        <v/>
+      </c>
+      <c r="G33" s="4">
+        <f>IF(D33=0,"",F33/D33)</f>
         <v/>
       </c>
     </row>
@@ -1294,11 +1350,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
@@ -1388,601 +1444,601 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>260</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Rental Income</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1350000</v>
+        <v>157000</v>
       </c>
       <c r="D2" t="n">
-        <v>1350000</v>
+        <v>157000</v>
       </c>
       <c r="E2" t="n">
-        <v>1350000</v>
+        <v>157000</v>
       </c>
       <c r="F2" t="n">
-        <v>1350000</v>
+        <v>157000</v>
       </c>
       <c r="G2" t="n">
-        <v>1350000</v>
+        <v>157000</v>
       </c>
       <c r="H2" t="n">
-        <v>1350000</v>
+        <v>157000</v>
       </c>
       <c r="I2" t="n">
-        <v>1350000</v>
+        <v>157000</v>
       </c>
       <c r="J2" t="n">
-        <v>1350000</v>
+        <v>157000</v>
       </c>
       <c r="K2" t="n">
-        <v>1350000</v>
+        <v>157000</v>
       </c>
       <c r="L2" t="n">
-        <v>1350000</v>
+        <v>157000</v>
       </c>
       <c r="M2" t="n">
-        <v>1350000</v>
+        <v>157000</v>
       </c>
       <c r="N2" t="n">
-        <v>1350000</v>
+        <v>157000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>270</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Other Revenue</t>
+          <t>Interest Income</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>85000</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>85000</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>85000</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>85000</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>85000</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>85000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>85000</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>85000</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>85000</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>85000</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>85000</v>
       </c>
       <c r="N3" t="n">
-        <v>0</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>275</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Interest Income</t>
+          <t>Dividend &amp; Portfolio Income</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1500</v>
+        <v>3800000</v>
       </c>
       <c r="D4" t="n">
-        <v>1500</v>
+        <v>3800000</v>
       </c>
       <c r="E4" t="n">
-        <v>1500</v>
+        <v>3800000</v>
       </c>
       <c r="F4" t="n">
-        <v>1500</v>
+        <v>3800000</v>
       </c>
       <c r="G4" t="n">
-        <v>1500</v>
+        <v>3800000</v>
       </c>
       <c r="H4" t="n">
-        <v>1500</v>
+        <v>3800000</v>
       </c>
       <c r="I4" t="n">
-        <v>1500</v>
+        <v>3800000</v>
       </c>
       <c r="J4" t="n">
-        <v>1500</v>
+        <v>3800000</v>
       </c>
       <c r="K4" t="n">
-        <v>1500</v>
+        <v>3800000</v>
       </c>
       <c r="L4" t="n">
-        <v>1500</v>
+        <v>3800000</v>
       </c>
       <c r="M4" t="n">
-        <v>1500</v>
+        <v>3800000</v>
       </c>
       <c r="N4" t="n">
-        <v>1500</v>
+        <v>3800000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>477</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold</t>
+          <t>Salaries - Office &amp; Household Staff</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>600000</v>
+        <v>420000</v>
       </c>
       <c r="D5" t="n">
-        <v>600000</v>
+        <v>420000</v>
       </c>
       <c r="E5" t="n">
-        <v>600000</v>
+        <v>420000</v>
       </c>
       <c r="F5" t="n">
-        <v>600000</v>
+        <v>420000</v>
       </c>
       <c r="G5" t="n">
-        <v>600000</v>
+        <v>420000</v>
       </c>
       <c r="H5" t="n">
-        <v>600000</v>
+        <v>420000</v>
       </c>
       <c r="I5" t="n">
-        <v>600000</v>
+        <v>420000</v>
       </c>
       <c r="J5" t="n">
-        <v>600000</v>
+        <v>420000</v>
       </c>
       <c r="K5" t="n">
-        <v>600000</v>
+        <v>420000</v>
       </c>
       <c r="L5" t="n">
-        <v>600000</v>
+        <v>420000</v>
       </c>
       <c r="M5" t="n">
-        <v>600000</v>
+        <v>420000</v>
       </c>
       <c r="N5" t="n">
-        <v>600000</v>
+        <v>420000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>425</t>
+          <t>478</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Freight &amp; Courier</t>
+          <t>MPF Contributions</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="D6" t="n">
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="E6" t="n">
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="F6" t="n">
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="G6" t="n">
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="H6" t="n">
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="I6" t="n">
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="J6" t="n">
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="K6" t="n">
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="L6" t="n">
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="M6" t="n">
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="N6" t="n">
-        <v>18000</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>445</t>
+          <t>471</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Utilities - Electricity</t>
+          <t>Property Management Fees</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>4800</v>
+        <v>18000</v>
       </c>
       <c r="D7" t="n">
-        <v>4800</v>
+        <v>18000</v>
       </c>
       <c r="E7" t="n">
-        <v>4800</v>
+        <v>18000</v>
       </c>
       <c r="F7" t="n">
-        <v>4800</v>
+        <v>18000</v>
       </c>
       <c r="G7" t="n">
-        <v>4800</v>
+        <v>18000</v>
       </c>
       <c r="H7" t="n">
-        <v>4800</v>
+        <v>18000</v>
       </c>
       <c r="I7" t="n">
-        <v>4800</v>
+        <v>18000</v>
       </c>
       <c r="J7" t="n">
-        <v>4800</v>
+        <v>18000</v>
       </c>
       <c r="K7" t="n">
-        <v>4800</v>
+        <v>18000</v>
       </c>
       <c r="L7" t="n">
-        <v>4800</v>
+        <v>18000</v>
       </c>
       <c r="M7" t="n">
-        <v>4800</v>
+        <v>18000</v>
       </c>
       <c r="N7" t="n">
-        <v>4800</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>469</t>
+          <t>473</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Rent</t>
+          <t>Property Repairs &amp; Maintenance</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>80000</v>
+        <v>3000</v>
       </c>
       <c r="D8" t="n">
-        <v>80000</v>
+        <v>3000</v>
       </c>
       <c r="E8" t="n">
-        <v>80000</v>
+        <v>3000</v>
       </c>
       <c r="F8" t="n">
-        <v>80000</v>
+        <v>3000</v>
       </c>
       <c r="G8" t="n">
-        <v>80000</v>
+        <v>3000</v>
       </c>
       <c r="H8" t="n">
-        <v>80000</v>
+        <v>3000</v>
       </c>
       <c r="I8" t="n">
-        <v>80000</v>
+        <v>3000</v>
       </c>
       <c r="J8" t="n">
-        <v>80000</v>
+        <v>3000</v>
       </c>
       <c r="K8" t="n">
-        <v>80000</v>
+        <v>3000</v>
       </c>
       <c r="L8" t="n">
-        <v>80000</v>
+        <v>3000</v>
       </c>
       <c r="M8" t="n">
-        <v>80000</v>
+        <v>3000</v>
       </c>
       <c r="N8" t="n">
-        <v>80000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>471</t>
+          <t>475</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Building Management Fees</t>
+          <t>Building Management &amp; Government Rates</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>6800</v>
+        <v>11600</v>
       </c>
       <c r="D9" t="n">
-        <v>6800</v>
+        <v>11600</v>
       </c>
       <c r="E9" t="n">
-        <v>6800</v>
+        <v>11600</v>
       </c>
       <c r="F9" t="n">
-        <v>6800</v>
+        <v>11600</v>
       </c>
       <c r="G9" t="n">
-        <v>6800</v>
+        <v>11600</v>
       </c>
       <c r="H9" t="n">
-        <v>6800</v>
+        <v>11600</v>
       </c>
       <c r="I9" t="n">
-        <v>6800</v>
+        <v>11600</v>
       </c>
       <c r="J9" t="n">
-        <v>6800</v>
+        <v>11600</v>
       </c>
       <c r="K9" t="n">
-        <v>6800</v>
+        <v>11600</v>
       </c>
       <c r="L9" t="n">
-        <v>6800</v>
+        <v>11600</v>
       </c>
       <c r="M9" t="n">
-        <v>6800</v>
+        <v>11600</v>
       </c>
       <c r="N9" t="n">
-        <v>6800</v>
+        <v>11600</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>473</t>
+          <t>481</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>School &amp; Tuition Fees</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2000</v>
+        <v>286000</v>
       </c>
       <c r="D10" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>2000</v>
+        <v>312000</v>
       </c>
       <c r="K10" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>477</t>
+          <t>493</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Salaries</t>
+          <t>Travel &amp; Aviation Charter</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>432000</v>
+        <v>125000</v>
       </c>
       <c r="D11" t="n">
-        <v>432000</v>
+        <v>125000</v>
       </c>
       <c r="E11" t="n">
-        <v>432000</v>
+        <v>125000</v>
       </c>
       <c r="F11" t="n">
-        <v>432000</v>
+        <v>125000</v>
       </c>
       <c r="G11" t="n">
-        <v>432000</v>
+        <v>125000</v>
       </c>
       <c r="H11" t="n">
-        <v>432000</v>
+        <v>125000</v>
       </c>
       <c r="I11" t="n">
-        <v>432000</v>
+        <v>125000</v>
       </c>
       <c r="J11" t="n">
-        <v>432000</v>
+        <v>125000</v>
       </c>
       <c r="K11" t="n">
-        <v>432000</v>
+        <v>125000</v>
       </c>
       <c r="L11" t="n">
-        <v>432000</v>
+        <v>125000</v>
       </c>
       <c r="M11" t="n">
-        <v>432000</v>
+        <v>125000</v>
       </c>
       <c r="N11" t="n">
-        <v>432000</v>
+        <v>125000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>478</t>
+          <t>433</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>MPF Contributions</t>
+          <t>Insurance</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>26400</v>
+        <v>67000</v>
       </c>
       <c r="D12" t="n">
-        <v>26400</v>
+        <v>19000</v>
       </c>
       <c r="E12" t="n">
-        <v>26400</v>
+        <v>19000</v>
       </c>
       <c r="F12" t="n">
-        <v>26400</v>
+        <v>19000</v>
       </c>
       <c r="G12" t="n">
-        <v>26400</v>
+        <v>19000</v>
       </c>
       <c r="H12" t="n">
-        <v>26400</v>
+        <v>19000</v>
       </c>
       <c r="I12" t="n">
-        <v>26400</v>
+        <v>19000</v>
       </c>
       <c r="J12" t="n">
-        <v>26400</v>
+        <v>19000</v>
       </c>
       <c r="K12" t="n">
-        <v>26400</v>
+        <v>19000</v>
       </c>
       <c r="L12" t="n">
-        <v>26400</v>
+        <v>19000</v>
       </c>
       <c r="M12" t="n">
-        <v>26400</v>
+        <v>19000</v>
       </c>
       <c r="N12" t="n">
-        <v>26400</v>
+        <v>19000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>412</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Bank Fees</t>
+          <t>Legal, Tax &amp; Audit Fees</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>450</v>
+        <v>28000</v>
       </c>
       <c r="D13" t="n">
-        <v>450</v>
+        <v>28000</v>
       </c>
       <c r="E13" t="n">
-        <v>450</v>
+        <v>148000</v>
       </c>
       <c r="F13" t="n">
-        <v>450</v>
+        <v>28000</v>
       </c>
       <c r="G13" t="n">
-        <v>450</v>
+        <v>28000</v>
       </c>
       <c r="H13" t="n">
-        <v>450</v>
+        <v>28000</v>
       </c>
       <c r="I13" t="n">
-        <v>450</v>
+        <v>28000</v>
       </c>
       <c r="J13" t="n">
-        <v>450</v>
+        <v>28000</v>
       </c>
       <c r="K13" t="n">
-        <v>450</v>
+        <v>28000</v>
       </c>
       <c r="L13" t="n">
-        <v>450</v>
+        <v>28000</v>
       </c>
       <c r="M13" t="n">
-        <v>450</v>
+        <v>28000</v>
       </c>
       <c r="N13" t="n">
-        <v>450</v>
+        <v>28000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>412</t>
+          <t>455</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Consulting &amp; Accounting</t>
+          <t>Fund Management Fees</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>292500</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>45000</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>292500</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
@@ -1991,7 +2047,7 @@
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>292500</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -2000,7 +2056,7 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>0</v>
+        <v>292500</v>
       </c>
       <c r="M14" t="n">
         <v>0</v>
@@ -2012,97 +2068,97 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>429</t>
+          <t>404</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>General Expenses</t>
+          <t>Bank Fees</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2500</v>
+        <v>900</v>
       </c>
       <c r="D15" t="n">
-        <v>2500</v>
+        <v>900</v>
       </c>
       <c r="E15" t="n">
-        <v>2500</v>
+        <v>900</v>
       </c>
       <c r="F15" t="n">
-        <v>2500</v>
+        <v>900</v>
       </c>
       <c r="G15" t="n">
-        <v>2500</v>
+        <v>900</v>
       </c>
       <c r="H15" t="n">
-        <v>2500</v>
+        <v>900</v>
       </c>
       <c r="I15" t="n">
-        <v>2500</v>
+        <v>900</v>
       </c>
       <c r="J15" t="n">
-        <v>2500</v>
+        <v>900</v>
       </c>
       <c r="K15" t="n">
-        <v>2500</v>
+        <v>900</v>
       </c>
       <c r="L15" t="n">
-        <v>2500</v>
+        <v>900</v>
       </c>
       <c r="M15" t="n">
-        <v>2500</v>
+        <v>900</v>
       </c>
       <c r="N15" t="n">
-        <v>2500</v>
+        <v>900</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>433</t>
+          <t>429</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Insurance</t>
+          <t>General Office Expenses</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>28800</v>
+        <v>9000</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>9000</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>9000</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>9000</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>9000</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>9000</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>9000</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>9000</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>9000</v>
       </c>
       <c r="L16" t="n">
-        <v>0</v>
+        <v>9000</v>
       </c>
       <c r="M16" t="n">
-        <v>0</v>
+        <v>9000</v>
       </c>
       <c r="N16" t="n">
-        <v>0</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="17">
@@ -2117,40 +2173,40 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>12700</v>
+        <v>3200</v>
       </c>
       <c r="D17" t="n">
-        <v>12700</v>
+        <v>3200</v>
       </c>
       <c r="E17" t="n">
-        <v>12700</v>
+        <v>3200</v>
       </c>
       <c r="F17" t="n">
-        <v>12700</v>
+        <v>3200</v>
       </c>
       <c r="G17" t="n">
-        <v>12700</v>
+        <v>3200</v>
       </c>
       <c r="H17" t="n">
-        <v>12700</v>
+        <v>3200</v>
       </c>
       <c r="I17" t="n">
-        <v>12700</v>
+        <v>3200</v>
       </c>
       <c r="J17" t="n">
-        <v>12700</v>
+        <v>3200</v>
       </c>
       <c r="K17" t="n">
-        <v>12700</v>
+        <v>3200</v>
       </c>
       <c r="L17" t="n">
-        <v>12700</v>
+        <v>3200</v>
       </c>
       <c r="M17" t="n">
-        <v>12700</v>
+        <v>3200</v>
       </c>
       <c r="N17" t="n">
-        <v>12700</v>
+        <v>3200</v>
       </c>
     </row>
     <row r="18">
@@ -2165,135 +2221,87 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1900</v>
+        <v>2400</v>
       </c>
       <c r="D18" t="n">
-        <v>1900</v>
+        <v>2400</v>
       </c>
       <c r="E18" t="n">
-        <v>1900</v>
+        <v>2400</v>
       </c>
       <c r="F18" t="n">
-        <v>1900</v>
+        <v>2400</v>
       </c>
       <c r="G18" t="n">
-        <v>1900</v>
+        <v>2400</v>
       </c>
       <c r="H18" t="n">
-        <v>1900</v>
+        <v>2400</v>
       </c>
       <c r="I18" t="n">
-        <v>1900</v>
+        <v>2400</v>
       </c>
       <c r="J18" t="n">
-        <v>1900</v>
+        <v>2400</v>
       </c>
       <c r="K18" t="n">
-        <v>1900</v>
+        <v>2400</v>
       </c>
       <c r="L18" t="n">
-        <v>1900</v>
+        <v>2400</v>
       </c>
       <c r="M18" t="n">
-        <v>1900</v>
+        <v>2400</v>
       </c>
       <c r="N18" t="n">
-        <v>1900</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>493</t>
+          <t>497</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Travel - Local &amp; Cross-border</t>
+          <t>Foreign Exchange Gain/Loss</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>4000</v>
+        <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>4000</v>
+        <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>4000</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>4000</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>4000</v>
+        <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>4000</v>
+        <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>4000</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>4000</v>
+        <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>4000</v>
+        <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>4000</v>
+        <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>4000</v>
+        <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>497</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Foreign Exchange Gain/Loss</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2308,11 +2316,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -2384,493 +2392,493 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>260</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Rental Income</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1337050</v>
+        <v>157000</v>
       </c>
       <c r="D2" t="n">
-        <v>1288980</v>
+        <v>157000</v>
       </c>
       <c r="E2" t="n">
-        <v>1332450</v>
+        <v>157000</v>
       </c>
       <c r="F2" t="n">
-        <v>1436050</v>
+        <v>157000</v>
       </c>
       <c r="G2" t="n">
-        <v>1480030</v>
+        <v>157000</v>
       </c>
       <c r="H2" t="n">
-        <v>1351400</v>
+        <v>157000</v>
       </c>
       <c r="I2" t="n">
-        <v>1456710</v>
+        <v>157000</v>
       </c>
       <c r="J2" t="n">
-        <v>1334750</v>
+        <v>157000</v>
       </c>
       <c r="K2" t="n">
-        <v>1460040</v>
+        <v>157000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>270</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Other Revenue</t>
+          <t>Interest Income</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>75992</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>92788</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>70772</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>89138</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>81251</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>70651</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>71843</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>75602</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>75748</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>275</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Interest Income</t>
+          <t>Dividend &amp; Portfolio Income</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1657</v>
+        <v>3553000</v>
       </c>
       <c r="D4" t="n">
-        <v>1580</v>
+        <v>3775000</v>
       </c>
       <c r="E4" t="n">
-        <v>1638</v>
+        <v>3815000</v>
       </c>
       <c r="F4" t="n">
-        <v>1107</v>
+        <v>3776000</v>
       </c>
       <c r="G4" t="n">
-        <v>1315</v>
+        <v>3700000</v>
       </c>
       <c r="H4" t="n">
-        <v>1782</v>
+        <v>3784000</v>
       </c>
       <c r="I4" t="n">
-        <v>1223</v>
+        <v>3680000</v>
       </c>
       <c r="J4" t="n">
-        <v>1162</v>
+        <v>3703000</v>
       </c>
       <c r="K4" t="n">
-        <v>1149</v>
+        <v>3554000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>477</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cost of Goods Sold</t>
+          <t>Salaries - Office &amp; Household Staff</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>618094.9</v>
+        <v>420000</v>
       </c>
       <c r="D5" t="n">
-        <v>599650.8100000001</v>
+        <v>420000</v>
       </c>
       <c r="E5" t="n">
-        <v>663247.4300000001</v>
+        <v>420000</v>
       </c>
       <c r="F5" t="n">
-        <v>550908.84</v>
+        <v>420000</v>
       </c>
       <c r="G5" t="n">
-        <v>583486.89</v>
+        <v>420000</v>
       </c>
       <c r="H5" t="n">
-        <v>670807.5</v>
+        <v>420000</v>
       </c>
       <c r="I5" t="n">
-        <v>600922.9300000001</v>
+        <v>420000</v>
       </c>
       <c r="J5" t="n">
-        <v>613779.46</v>
+        <v>420000</v>
       </c>
       <c r="K5" t="n">
-        <v>635229.6</v>
+        <v>420000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>425</t>
+          <t>478</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Freight &amp; Courier</t>
+          <t>MPF Contributions</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>22350</v>
+        <v>15000</v>
       </c>
       <c r="D6" t="n">
-        <v>16290</v>
+        <v>15000</v>
       </c>
       <c r="E6" t="n">
-        <v>22485</v>
+        <v>15000</v>
       </c>
       <c r="F6" t="n">
-        <v>16335</v>
+        <v>15000</v>
       </c>
       <c r="G6" t="n">
-        <v>11760</v>
+        <v>15000</v>
       </c>
       <c r="H6" t="n">
-        <v>16290</v>
+        <v>15000</v>
       </c>
       <c r="I6" t="n">
-        <v>23925</v>
+        <v>15000</v>
       </c>
       <c r="J6" t="n">
-        <v>33180</v>
+        <v>15000</v>
       </c>
       <c r="K6" t="n">
-        <v>27660</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>445</t>
+          <t>471</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Utilities - Electricity</t>
+          <t>Property Management Fees</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>4388</v>
+        <v>17300</v>
       </c>
       <c r="D7" t="n">
-        <v>4342</v>
+        <v>17300</v>
       </c>
       <c r="E7" t="n">
-        <v>4363</v>
+        <v>23200</v>
       </c>
       <c r="F7" t="n">
-        <v>4006</v>
+        <v>23200</v>
       </c>
       <c r="G7" t="n">
-        <v>4293</v>
+        <v>23200</v>
       </c>
       <c r="H7" t="n">
-        <v>5981</v>
+        <v>23200</v>
       </c>
       <c r="I7" t="n">
-        <v>5775</v>
+        <v>23200</v>
       </c>
       <c r="J7" t="n">
-        <v>5705</v>
+        <v>17300</v>
       </c>
       <c r="K7" t="n">
-        <v>5819</v>
+        <v>23200</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>469</t>
+          <t>473</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Rent</t>
+          <t>Property Repairs &amp; Maintenance</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>80000</v>
+        <v>1100</v>
       </c>
       <c r="D8" t="n">
-        <v>80000</v>
+        <v>1800</v>
       </c>
       <c r="E8" t="n">
-        <v>80000</v>
+        <v>2600</v>
       </c>
       <c r="F8" t="n">
-        <v>80000</v>
+        <v>1500</v>
       </c>
       <c r="G8" t="n">
-        <v>80000</v>
+        <v>2300</v>
       </c>
       <c r="H8" t="n">
-        <v>80000</v>
+        <v>1800</v>
       </c>
       <c r="I8" t="n">
-        <v>80000</v>
+        <v>39600</v>
       </c>
       <c r="J8" t="n">
-        <v>92000</v>
+        <v>2300</v>
       </c>
       <c r="K8" t="n">
-        <v>92000</v>
+        <v>12300</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>471</t>
+          <t>475</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Building Management Fees</t>
+          <t>Building Management &amp; Government Rates</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>6800</v>
+        <v>11600</v>
       </c>
       <c r="D9" t="n">
-        <v>6800</v>
+        <v>11600</v>
       </c>
       <c r="E9" t="n">
-        <v>6800</v>
+        <v>11600</v>
       </c>
       <c r="F9" t="n">
-        <v>6800</v>
+        <v>11600</v>
       </c>
       <c r="G9" t="n">
-        <v>6800</v>
+        <v>11600</v>
       </c>
       <c r="H9" t="n">
-        <v>8000</v>
+        <v>12800</v>
       </c>
       <c r="I9" t="n">
-        <v>8000</v>
+        <v>12800</v>
       </c>
       <c r="J9" t="n">
-        <v>8000</v>
+        <v>12800</v>
       </c>
       <c r="K9" t="n">
-        <v>8000</v>
+        <v>12800</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>473</t>
+          <t>481</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Repairs &amp; Maintenance</t>
+          <t>School &amp; Tuition Fees</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1200</v>
+        <v>286000</v>
       </c>
       <c r="D10" t="n">
-        <v>1800</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>1900</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>1600</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>1800</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>39500</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>1700</v>
+        <v>318000</v>
       </c>
       <c r="K10" t="n">
-        <v>10800</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>477</t>
+          <t>493</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Salaries</t>
+          <t>Travel &amp; Aviation Charter</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>432000</v>
+        <v>107000</v>
       </c>
       <c r="D11" t="n">
-        <v>432000</v>
+        <v>119000</v>
       </c>
       <c r="E11" t="n">
-        <v>432000</v>
+        <v>143000</v>
       </c>
       <c r="F11" t="n">
-        <v>432000</v>
+        <v>146000</v>
       </c>
       <c r="G11" t="n">
-        <v>432000</v>
+        <v>152000</v>
       </c>
       <c r="H11" t="n">
-        <v>432000</v>
+        <v>88000</v>
       </c>
       <c r="I11" t="n">
-        <v>432000</v>
+        <v>135000</v>
       </c>
       <c r="J11" t="n">
-        <v>432000</v>
+        <v>89000</v>
       </c>
       <c r="K11" t="n">
-        <v>432000</v>
+        <v>148000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>478</t>
+          <t>433</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>MPF Contributions</t>
+          <t>Insurance</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>26400</v>
+        <v>67085.5</v>
       </c>
       <c r="D12" t="n">
-        <v>26400</v>
+        <v>19134.5</v>
       </c>
       <c r="E12" t="n">
-        <v>26400</v>
+        <v>19159</v>
       </c>
       <c r="F12" t="n">
-        <v>26400</v>
+        <v>19110</v>
       </c>
       <c r="G12" t="n">
-        <v>26400</v>
+        <v>19085.5</v>
       </c>
       <c r="H12" t="n">
-        <v>26400</v>
+        <v>19134.5</v>
       </c>
       <c r="I12" t="n">
-        <v>26400</v>
+        <v>19159</v>
       </c>
       <c r="J12" t="n">
-        <v>26400</v>
+        <v>19134.5</v>
       </c>
       <c r="K12" t="n">
-        <v>26400</v>
+        <v>19110</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>412</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Bank Fees</t>
+          <t>Legal, Tax &amp; Audit Fees</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>570</v>
+        <v>28000</v>
       </c>
       <c r="D13" t="n">
-        <v>570</v>
+        <v>28000</v>
       </c>
       <c r="E13" t="n">
-        <v>570</v>
+        <v>148000</v>
       </c>
       <c r="F13" t="n">
-        <v>570</v>
+        <v>28000</v>
       </c>
       <c r="G13" t="n">
-        <v>570</v>
+        <v>28000</v>
       </c>
       <c r="H13" t="n">
-        <v>570</v>
+        <v>28000</v>
       </c>
       <c r="I13" t="n">
-        <v>570</v>
+        <v>28000</v>
       </c>
       <c r="J13" t="n">
-        <v>570</v>
+        <v>28000</v>
       </c>
       <c r="K13" t="n">
-        <v>570</v>
+        <v>28000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>412</t>
+          <t>455</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Consulting &amp; Accounting</t>
+          <t>Fund Management Fees</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>292125</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>45000</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>292500</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
@@ -2879,7 +2887,7 @@
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>293250</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -2891,79 +2899,79 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>429</t>
+          <t>404</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>General Expenses</t>
+          <t>Bank Fees</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1400</v>
+        <v>420</v>
       </c>
       <c r="D15" t="n">
-        <v>1600</v>
+        <v>570</v>
       </c>
       <c r="E15" t="n">
-        <v>1300</v>
+        <v>420</v>
       </c>
       <c r="F15" t="n">
-        <v>2400</v>
+        <v>270</v>
       </c>
       <c r="G15" t="n">
-        <v>1500</v>
+        <v>720</v>
       </c>
       <c r="H15" t="n">
-        <v>1200</v>
+        <v>270</v>
       </c>
       <c r="I15" t="n">
-        <v>3100</v>
+        <v>570</v>
       </c>
       <c r="J15" t="n">
-        <v>3100</v>
+        <v>420</v>
       </c>
       <c r="K15" t="n">
-        <v>2500</v>
+        <v>270</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>433</t>
+          <t>429</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Insurance</t>
+          <t>General Office Expenses</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>28800</v>
+        <v>10800</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>9900</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>7400</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>9000</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>9900</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>6400</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>10200</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>6400</v>
       </c>
     </row>
     <row r="17">
@@ -2978,31 +2986,31 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>12615.5</v>
+        <v>3150</v>
       </c>
       <c r="D17" t="n">
-        <v>12644.5</v>
+        <v>3150</v>
       </c>
       <c r="E17" t="n">
-        <v>12659</v>
+        <v>3150</v>
       </c>
       <c r="F17" t="n">
-        <v>12630</v>
+        <v>3150</v>
       </c>
       <c r="G17" t="n">
-        <v>12615.5</v>
+        <v>3150</v>
       </c>
       <c r="H17" t="n">
-        <v>12644.5</v>
+        <v>3150</v>
       </c>
       <c r="I17" t="n">
-        <v>12659</v>
+        <v>3150</v>
       </c>
       <c r="J17" t="n">
-        <v>12644.5</v>
+        <v>3150</v>
       </c>
       <c r="K17" t="n">
-        <v>12630</v>
+        <v>3150</v>
       </c>
     </row>
     <row r="18">
@@ -3017,109 +3025,70 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1880</v>
+        <v>2380</v>
       </c>
       <c r="D18" t="n">
-        <v>1880</v>
+        <v>2380</v>
       </c>
       <c r="E18" t="n">
-        <v>1880</v>
+        <v>2380</v>
       </c>
       <c r="F18" t="n">
-        <v>1880</v>
+        <v>2380</v>
       </c>
       <c r="G18" t="n">
-        <v>1880</v>
+        <v>2380</v>
       </c>
       <c r="H18" t="n">
-        <v>1880</v>
+        <v>2380</v>
       </c>
       <c r="I18" t="n">
-        <v>1880</v>
+        <v>2380</v>
       </c>
       <c r="J18" t="n">
-        <v>1880</v>
+        <v>2380</v>
       </c>
       <c r="K18" t="n">
-        <v>1880</v>
+        <v>2380</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>493</t>
+          <t>497</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Travel - Local &amp; Cross-border</t>
+          <t>Foreign Exchange Gain/Loss</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2400</v>
+        <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>2300</v>
+        <v>750</v>
       </c>
       <c r="E19" t="n">
-        <v>3200</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>4500</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>2100</v>
+        <v>-375</v>
       </c>
       <c r="H19" t="n">
-        <v>3300</v>
+        <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>3300</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>5400</v>
+        <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>2300</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>497</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Foreign Exchange Gain/Loss</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>-297.16</v>
-      </c>
-      <c r="D20" t="n">
-        <v>2789.3</v>
-      </c>
-      <c r="E20" t="n">
-        <v>2615.4</v>
-      </c>
-      <c r="F20" t="n">
-        <v>-952.83</v>
-      </c>
-      <c r="G20" t="n">
-        <v>-2532.42</v>
-      </c>
-      <c r="H20" t="n">
-        <v>1237.38</v>
-      </c>
-      <c r="I20" t="n">
-        <v>3477.4</v>
-      </c>
-      <c r="J20" t="n">
-        <v>1001.4</v>
-      </c>
-      <c r="K20" t="n">
-        <v>-1306.03</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>